<commit_message>
Migrate pricing to Excel master and remove CSV pricing file
</commit_message>
<xml_diff>
--- a/data/Factura Proforma.xlsx
+++ b/data/Factura Proforma.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mauriciogonzalez/Documents/export_commercial_ai/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{DCC4FB16-492E-B04C-8E77-4259637544AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A0F8180D-BA92-FC43-A706-6EDF9B3192C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4420" yWindow="660" windowWidth="23260" windowHeight="13900" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="18460" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Orden" sheetId="1" r:id="rId1"/>
@@ -91,7 +91,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="118" uniqueCount="73">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="129" uniqueCount="74">
   <si>
     <t>FACTURA PROFORMA</t>
   </si>
@@ -279,9 +279,6 @@
     <t>Descripcion</t>
   </si>
   <si>
-    <t>LISTA</t>
-  </si>
-  <si>
     <t>AUCCN</t>
   </si>
   <si>
@@ -297,9 +294,6 @@
     <t>Lista</t>
   </si>
   <si>
-    <t>LISTA P</t>
-  </si>
-  <si>
     <t>AUBRAVO</t>
   </si>
   <si>
@@ -310,6 +304,15 @@
   </si>
   <si>
     <t>AV. WINSTON CHURCHIL ESQ. ANGEL</t>
+  </si>
+  <si>
+    <t>LISTA_PRECIOS</t>
+  </si>
+  <si>
+    <t>ORIGEN</t>
+  </si>
+  <si>
+    <t>GUATEMALA</t>
   </si>
 </sst>
 </file>
@@ -644,7 +647,7 @@
     <xf numFmtId="165" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="84">
+  <cellXfs count="85">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="6" applyFont="1"/>
     <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -866,6 +869,9 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="13" fillId="0" borderId="4" xfId="8" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="9">
@@ -879,7 +885,41 @@
     <cellStyle name="Normal 3" xfId="2" xr:uid="{1A6DFAA5-2C19-462D-A953-FA9D01447442}"/>
     <cellStyle name="Porcentaje" xfId="6" builtinId="5"/>
   </cellStyles>
-  <dxfs count="30">
+  <dxfs count="31">
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <name val="Helvetica Neue"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="1" formatCode="0"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top/>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
     <dxf>
       <font>
         <b/>
@@ -1271,47 +1311,6 @@
         <top/>
         <bottom/>
       </border>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -1488,6 +1487,47 @@
         <top/>
         <bottom/>
       </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
   </dxfs>
   <tableStyles count="1" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16">
@@ -1700,59 +1740,60 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{8A94E3B6-9EAD-4329-8389-0ADCBCC848EA}" name="Tabla1" displayName="Tabla1" ref="A14:H42" totalsRowShown="0" headerRowDxfId="29" dataDxfId="27" headerRowBorderDxfId="28" tableBorderDxfId="26">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{8A94E3B6-9EAD-4329-8389-0ADCBCC848EA}" name="Tabla1" displayName="Tabla1" ref="A14:H42" totalsRowShown="0" headerRowDxfId="27" dataDxfId="25" headerRowBorderDxfId="26" tableBorderDxfId="24">
   <autoFilter ref="A14:H42" xr:uid="{8A94E3B6-9EAD-4329-8389-0ADCBCC848EA}"/>
   <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{520CA9FA-584B-4358-9B15-E654607E7AA3}" name="Código Interno" dataDxfId="25"/>
-    <tableColumn id="2" xr3:uid="{B5EE805F-D79D-4B18-9969-A438C10D73CB}" name="Código de Barra" dataDxfId="24">
+    <tableColumn id="1" xr3:uid="{520CA9FA-584B-4358-9B15-E654607E7AA3}" name="Código Interno" dataDxfId="23"/>
+    <tableColumn id="2" xr3:uid="{B5EE805F-D79D-4B18-9969-A438C10D73CB}" name="Código de Barra" dataDxfId="22">
       <calculatedColumnFormula>IFERROR(_xlfn.XLOOKUP(K15,Precios!K:K,Precios!I:I,0),"0")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{8E379099-A773-4C78-99DE-A30F428DCAA3}" name="Descripción del producto/servicio" dataDxfId="23"/>
-    <tableColumn id="5" xr3:uid="{3D35979A-292B-42DE-B9B7-4C01FAD4E4DB}" name="Cajas" dataDxfId="22"/>
-    <tableColumn id="6" xr3:uid="{1C8C5A17-73DF-4E24-BD8B-C3B44F70EC3B}" name="Piezas por Cj" dataDxfId="21"/>
-    <tableColumn id="7" xr3:uid="{4AC8BB4B-EFC3-40D6-BD2F-E267A391DA14}" name="Precio Unitario US$" dataDxfId="20"/>
-    <tableColumn id="8" xr3:uid="{8E18F1A5-A975-43AC-AC23-157590FF40C9}" name="Precio Caja US$" dataDxfId="19"/>
-    <tableColumn id="9" xr3:uid="{5EEA48C5-DAD6-467E-BE56-8D618AF7F476}" name="Precio Total" dataDxfId="18"/>
+    <tableColumn id="3" xr3:uid="{8E379099-A773-4C78-99DE-A30F428DCAA3}" name="Descripción del producto/servicio" dataDxfId="21"/>
+    <tableColumn id="5" xr3:uid="{3D35979A-292B-42DE-B9B7-4C01FAD4E4DB}" name="Cajas" dataDxfId="20"/>
+    <tableColumn id="6" xr3:uid="{1C8C5A17-73DF-4E24-BD8B-C3B44F70EC3B}" name="Piezas por Cj" dataDxfId="19"/>
+    <tableColumn id="7" xr3:uid="{4AC8BB4B-EFC3-40D6-BD2F-E267A391DA14}" name="Precio Unitario US$" dataDxfId="18"/>
+    <tableColumn id="8" xr3:uid="{8E18F1A5-A975-43AC-AC23-157590FF40C9}" name="Precio Caja US$" dataDxfId="17"/>
+    <tableColumn id="9" xr3:uid="{5EEA48C5-DAD6-467E-BE56-8D618AF7F476}" name="Precio Total" dataDxfId="16"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight16" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{8669CD56-B58B-4ACB-8B3C-F2934DCE7691}" name="Tabla2" displayName="Tabla2" ref="A1:F5" totalsRowShown="0" headerRowDxfId="17">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{8669CD56-B58B-4ACB-8B3C-F2934DCE7691}" name="Tabla2" displayName="Tabla2" ref="A1:F5" totalsRowShown="0" headerRowDxfId="30">
   <autoFilter ref="A1:F5" xr:uid="{8669CD56-B58B-4ACB-8B3C-F2934DCE7691}"/>
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{0D58B185-A9C1-48AD-B2F4-32DF9E217F13}" name="NIF:"/>
     <tableColumn id="2" xr3:uid="{33CBF84B-48C6-447A-BBF2-DD5AA8FCC61A}" name="Cliente"/>
     <tableColumn id="3" xr3:uid="{24888C6A-371D-47AF-9D61-4D5A564AB563}" name="DIRECCION"/>
-    <tableColumn id="4" xr3:uid="{54776D73-D261-4857-BA0D-C5404DB9B619}" name="Contacto:" dataDxfId="16"/>
+    <tableColumn id="4" xr3:uid="{54776D73-D261-4857-BA0D-C5404DB9B619}" name="Contacto:" dataDxfId="29"/>
     <tableColumn id="5" xr3:uid="{92F18AB8-E877-464C-B2B7-EB1E14CC628E}" name="NUMERO"/>
-    <tableColumn id="6" xr3:uid="{517F7E11-B7D8-4826-98B4-D4A8F078F50D}" name="LISTA P" dataDxfId="15"/>
+    <tableColumn id="6" xr3:uid="{517F7E11-B7D8-4826-98B4-D4A8F078F50D}" name="LISTA_PRECIOS" dataDxfId="28"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{9A4FE505-CC4B-404E-AD0E-A96422E28D9D}" name="Tabla3" displayName="Tabla3" ref="A1:L11" totalsRowShown="0" headerRowDxfId="14" dataDxfId="13" tableBorderDxfId="12" dataCellStyle="Moneda [0]">
-  <autoFilter ref="A1:L11" xr:uid="{9A4FE505-CC4B-404E-AD0E-A96422E28D9D}"/>
-  <tableColumns count="12">
-    <tableColumn id="1" xr3:uid="{DA0F2924-236B-47E9-A2A7-9191F873C793}" name="MARCA" dataDxfId="11"/>
-    <tableColumn id="2" xr3:uid="{D6ABD749-CE3A-429C-BE83-AC7C508C046F}" name="CODIGO" dataDxfId="10"/>
-    <tableColumn id="3" xr3:uid="{2839CEA5-BFD1-4AF4-9992-43115BB826C1}" name="Descripcion" dataDxfId="9"/>
-    <tableColumn id="4" xr3:uid="{66385BFB-7AC9-4F92-AEE8-3895D2EC51F5}" name="GRAMOS" dataDxfId="8"/>
-    <tableColumn id="5" xr3:uid="{791BE4D0-775A-4584-B7A9-A710D72CA463}" name="Precio CIF" dataDxfId="7" dataCellStyle="Moneda [0]"/>
-    <tableColumn id="6" xr3:uid="{7DC72C83-E4B3-4FA6-A4BB-7DFD7B7351DE}" name="Caja" dataDxfId="6" dataCellStyle="Moneda [0]"/>
-    <tableColumn id="7" xr3:uid="{E322D55A-4385-489C-B408-E5F854A495AF}" name="Pallet" dataDxfId="5" dataCellStyle="Moneda [0]"/>
-    <tableColumn id="11" xr3:uid="{B97156C5-49D3-4846-A5C8-ABD0A02AAA8D}" name="Precio CJ" dataDxfId="4">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{9A4FE505-CC4B-404E-AD0E-A96422E28D9D}" name="Tabla3" displayName="Tabla3" ref="A1:M11" totalsRowShown="0" headerRowDxfId="15" dataDxfId="14" tableBorderDxfId="13" dataCellStyle="Moneda [0]">
+  <autoFilter ref="A1:M11" xr:uid="{9A4FE505-CC4B-404E-AD0E-A96422E28D9D}"/>
+  <tableColumns count="13">
+    <tableColumn id="1" xr3:uid="{DA0F2924-236B-47E9-A2A7-9191F873C793}" name="MARCA" dataDxfId="12"/>
+    <tableColumn id="2" xr3:uid="{D6ABD749-CE3A-429C-BE83-AC7C508C046F}" name="CODIGO" dataDxfId="11"/>
+    <tableColumn id="3" xr3:uid="{2839CEA5-BFD1-4AF4-9992-43115BB826C1}" name="Descripcion" dataDxfId="10"/>
+    <tableColumn id="4" xr3:uid="{66385BFB-7AC9-4F92-AEE8-3895D2EC51F5}" name="GRAMOS" dataDxfId="9"/>
+    <tableColumn id="5" xr3:uid="{791BE4D0-775A-4584-B7A9-A710D72CA463}" name="Precio CIF" dataDxfId="8" dataCellStyle="Moneda [0]"/>
+    <tableColumn id="6" xr3:uid="{7DC72C83-E4B3-4FA6-A4BB-7DFD7B7351DE}" name="Caja" dataDxfId="7" dataCellStyle="Moneda [0]"/>
+    <tableColumn id="7" xr3:uid="{E322D55A-4385-489C-B408-E5F854A495AF}" name="Pallet" dataDxfId="6" dataCellStyle="Moneda [0]"/>
+    <tableColumn id="11" xr3:uid="{B97156C5-49D3-4846-A5C8-ABD0A02AAA8D}" name="Precio CJ" dataDxfId="5">
       <calculatedColumnFormula>E2*F2</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="12" xr3:uid="{2C02D87E-8CB1-49F8-A5BE-03855A6C1E9B}" name="COD BARRAS" dataDxfId="3"/>
-    <tableColumn id="13" xr3:uid="{E5AD99A8-D6B8-4E4D-B228-7FB94061B422}" name="LISTA" dataDxfId="2" dataCellStyle="Moneda [0]"/>
-    <tableColumn id="14" xr3:uid="{51631B47-0651-4FAD-9063-AA561FBD4C48}" name="Clave" dataDxfId="1" dataCellStyle="Moneda [0]">
-      <calculatedColumnFormula>_xlfn.CONCAT(Tabla3[[#This Row],[CODIGO]],Tabla3[[#This Row],[LISTA]])</calculatedColumnFormula>
+    <tableColumn id="12" xr3:uid="{2C02D87E-8CB1-49F8-A5BE-03855A6C1E9B}" name="COD BARRAS" dataDxfId="4"/>
+    <tableColumn id="13" xr3:uid="{E5AD99A8-D6B8-4E4D-B228-7FB94061B422}" name="LISTA_PRECIOS" dataDxfId="3" dataCellStyle="Moneda [0]"/>
+    <tableColumn id="14" xr3:uid="{51631B47-0651-4FAD-9063-AA561FBD4C48}" name="Clave" dataDxfId="2" dataCellStyle="Moneda [0]">
+      <calculatedColumnFormula>_xlfn.CONCAT(Tabla3[[#This Row],[CODIGO]],Tabla3[[#This Row],[LISTA_PRECIOS]])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="16" xr3:uid="{AC660C86-F1B8-4D6F-B5EA-B71D403A6C74}" name="Columna1" dataDxfId="0" dataCellStyle="Moneda [0]"/>
+    <tableColumn id="16" xr3:uid="{AC660C86-F1B8-4D6F-B5EA-B71D403A6C74}" name="Columna1" dataDxfId="1" dataCellStyle="Moneda [0]"/>
+    <tableColumn id="8" xr3:uid="{AC200EC2-556C-E346-8A2C-D4CB607D1887}" name="ORIGEN" dataDxfId="0" dataCellStyle="Moneda [0]"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2107,7 +2148,7 @@
       </c>
       <c r="B5" s="47">
         <f ca="1">TODAY()</f>
-        <v>46170</v>
+        <v>46171</v>
       </c>
       <c r="C5" s="41"/>
       <c r="D5" s="44"/>
@@ -2223,7 +2264,7 @@
       <c r="D12" s="58"/>
       <c r="E12" s="59"/>
       <c r="F12" s="52" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="G12" s="60" t="str">
         <f>_xlfn.XLOOKUP(B13,Clientes!A:A,Clientes!F:F,0)</f>
@@ -2274,7 +2315,7 @@
       </c>
       <c r="I14" s="82"/>
       <c r="K14" s="34" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.2">
@@ -2893,7 +2934,7 @@
     <col min="3" max="3" width="53.6640625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="17" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="11.83203125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11.5" style="11"/>
+    <col min="6" max="6" width="17.5" style="11" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.2">
@@ -2913,7 +2954,7 @@
         <v>51</v>
       </c>
       <c r="F1" s="19" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.2">
@@ -2930,10 +2971,10 @@
         <v>8</v>
       </c>
       <c r="E2" s="17" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="F2" s="11" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="3" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.2">
@@ -2950,10 +2991,10 @@
         <v>58</v>
       </c>
       <c r="E3" s="17" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="F3" s="11" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.2">
@@ -2968,10 +3009,10 @@
       </c>
       <c r="D4" s="15"/>
       <c r="E4" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="F4" s="11" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.2">
@@ -2979,10 +3020,10 @@
         <v>147006</v>
       </c>
       <c r="B5" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="C5" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="D5" s="15"/>
     </row>
@@ -2996,7 +3037,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{85ACCD81-FF74-4615-9937-AC8E05B80C69}">
-  <dimension ref="A1:L11"/>
+  <dimension ref="A1:M11"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="3" max="3" width="34.33203125" customWidth="1"/>
@@ -3004,11 +3045,13 @@
     <col min="5" max="5" width="15" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="14.1640625" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="14" style="11" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="15.83203125" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="24.83203125" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="34.6640625" customWidth="1"/>
+    <col min="13" max="13" width="12.83203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="17" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:13" ht="17" x14ac:dyDescent="0.2">
       <c r="A1" s="20" t="s">
         <v>26</v>
       </c>
@@ -3037,16 +3080,19 @@
         <v>47</v>
       </c>
       <c r="J1" s="30" t="s">
-        <v>62</v>
+        <v>71</v>
       </c>
       <c r="K1" s="30" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="L1" s="30" t="s">
         <v>52</v>
       </c>
-    </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M1" s="30" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A2" s="18" t="s">
         <v>33</v>
       </c>
@@ -3076,17 +3122,20 @@
         <v>658480001101</v>
       </c>
       <c r="J2" s="29" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="K2" s="29" t="str">
-        <f>_xlfn.CONCAT(Tabla3[[#This Row],[CODIGO]],Tabla3[[#This Row],[LISTA]])</f>
+        <f>_xlfn.CONCAT(Tabla3[[#This Row],[CODIGO]],Tabla3[[#This Row],[LISTA_PRECIOS]])</f>
         <v>504757AUCCN</v>
       </c>
       <c r="L2" s="29" t="s">
         <v>60</v>
       </c>
-    </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M2" s="84" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A3" s="21" t="s">
         <v>35</v>
       </c>
@@ -3116,17 +3165,20 @@
         <v>7441029500400</v>
       </c>
       <c r="J3" s="29" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="K3" s="10" t="str">
-        <f>_xlfn.CONCAT(Tabla3[[#This Row],[CODIGO]],Tabla3[[#This Row],[LISTA]])</f>
+        <f>_xlfn.CONCAT(Tabla3[[#This Row],[CODIGO]],Tabla3[[#This Row],[LISTA_PRECIOS]])</f>
         <v>505252AUCCN</v>
       </c>
       <c r="L3" s="29" t="s">
         <v>60</v>
       </c>
-    </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M3" s="84" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A4" s="21" t="s">
         <v>35</v>
       </c>
@@ -3156,17 +3208,20 @@
         <v>7441029556025</v>
       </c>
       <c r="J4" s="29" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="K4" s="10" t="str">
-        <f>_xlfn.CONCAT(Tabla3[[#This Row],[CODIGO]],Tabla3[[#This Row],[LISTA]])</f>
+        <f>_xlfn.CONCAT(Tabla3[[#This Row],[CODIGO]],Tabla3[[#This Row],[LISTA_PRECIOS]])</f>
         <v>1233AUCCN</v>
       </c>
       <c r="L4" s="29" t="s">
         <v>60</v>
       </c>
-    </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M4" s="84" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A5" s="21" t="s">
         <v>35</v>
       </c>
@@ -3196,17 +3251,20 @@
         <v>7441029507041</v>
       </c>
       <c r="J5" s="29" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="K5" s="10" t="str">
-        <f>_xlfn.CONCAT(Tabla3[[#This Row],[CODIGO]],Tabla3[[#This Row],[LISTA]])</f>
+        <f>_xlfn.CONCAT(Tabla3[[#This Row],[CODIGO]],Tabla3[[#This Row],[LISTA_PRECIOS]])</f>
         <v>24184AUCCN</v>
       </c>
       <c r="L5" s="29" t="s">
         <v>60</v>
       </c>
-    </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M5" s="84" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A6" s="22" t="s">
         <v>38</v>
       </c>
@@ -3236,17 +3294,20 @@
         <v>7441029500141</v>
       </c>
       <c r="J6" s="29" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="K6" s="26" t="str">
-        <f>_xlfn.CONCAT(Tabla3[[#This Row],[CODIGO]],Tabla3[[#This Row],[LISTA]])</f>
+        <f>_xlfn.CONCAT(Tabla3[[#This Row],[CODIGO]],Tabla3[[#This Row],[LISTA_PRECIOS]])</f>
         <v>5707AUCCN</v>
       </c>
       <c r="L6" s="29" t="s">
         <v>60</v>
       </c>
-    </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M6" s="84" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A7" s="21" t="s">
         <v>33</v>
       </c>
@@ -3276,17 +3337,20 @@
         <v>658480001101</v>
       </c>
       <c r="J7" s="10" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="K7" s="10" t="str">
-        <f>_xlfn.CONCAT(Tabla3[[#This Row],[CODIGO]],Tabla3[[#This Row],[LISTA]])</f>
+        <f>_xlfn.CONCAT(Tabla3[[#This Row],[CODIGO]],Tabla3[[#This Row],[LISTA_PRECIOS]])</f>
         <v>504757AUBRAVO</v>
       </c>
       <c r="L7" s="10" t="s">
         <v>53</v>
       </c>
-    </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M7" s="84" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A8" s="21" t="s">
         <v>35</v>
       </c>
@@ -3316,17 +3380,20 @@
         <v>7441029500400</v>
       </c>
       <c r="J8" s="10" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="K8" s="10" t="str">
-        <f>_xlfn.CONCAT(Tabla3[[#This Row],[CODIGO]],Tabla3[[#This Row],[LISTA]])</f>
+        <f>_xlfn.CONCAT(Tabla3[[#This Row],[CODIGO]],Tabla3[[#This Row],[LISTA_PRECIOS]])</f>
         <v>505252AUBRAVO</v>
       </c>
       <c r="L8" s="10" t="s">
         <v>53</v>
       </c>
-    </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M8" s="84" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A9" s="21" t="s">
         <v>35</v>
       </c>
@@ -3356,17 +3423,20 @@
         <v>7441029556025</v>
       </c>
       <c r="J9" s="10" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="K9" s="10" t="str">
-        <f>_xlfn.CONCAT(Tabla3[[#This Row],[CODIGO]],Tabla3[[#This Row],[LISTA]])</f>
+        <f>_xlfn.CONCAT(Tabla3[[#This Row],[CODIGO]],Tabla3[[#This Row],[LISTA_PRECIOS]])</f>
         <v>1233AUBRAVO</v>
       </c>
       <c r="L9" s="10" t="s">
         <v>53</v>
       </c>
-    </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M9" s="84" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A10" s="21" t="s">
         <v>35</v>
       </c>
@@ -3396,17 +3466,20 @@
         <v>7441029507041</v>
       </c>
       <c r="J10" s="10" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="K10" s="10" t="str">
-        <f>_xlfn.CONCAT(Tabla3[[#This Row],[CODIGO]],Tabla3[[#This Row],[LISTA]])</f>
+        <f>_xlfn.CONCAT(Tabla3[[#This Row],[CODIGO]],Tabla3[[#This Row],[LISTA_PRECIOS]])</f>
         <v>24184AUBRAVO</v>
       </c>
       <c r="L10" s="10" t="s">
         <v>53</v>
       </c>
-    </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M10" s="84" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="11" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A11" s="22" t="s">
         <v>38</v>
       </c>
@@ -3436,14 +3509,17 @@
         <v>7441029500141</v>
       </c>
       <c r="J11" s="10" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="K11" s="26" t="str">
-        <f>_xlfn.CONCAT(Tabla3[[#This Row],[CODIGO]],Tabla3[[#This Row],[LISTA]])</f>
+        <f>_xlfn.CONCAT(Tabla3[[#This Row],[CODIGO]],Tabla3[[#This Row],[LISTA_PRECIOS]])</f>
         <v>5707AUBRAVO</v>
       </c>
       <c r="L11" s="10" t="s">
         <v>53</v>
+      </c>
+      <c r="M11" s="84" t="s">
+        <v>73</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Generate separate proformas by origin
</commit_message>
<xml_diff>
--- a/data/Factura Proforma.xlsx
+++ b/data/Factura Proforma.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mauriciogonzalez/Documents/export_commercial_ai/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A0F8180D-BA92-FC43-A706-6EDF9B3192C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AA489619-14CF-1046-9BA5-F7B9ED22870F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="18460" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4420" yWindow="660" windowWidth="24980" windowHeight="17060" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Orden" sheetId="1" r:id="rId1"/>
@@ -852,6 +852,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="1" fontId="13" fillId="0" borderId="4" xfId="8" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="16" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -869,9 +872,6 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="13" fillId="0" borderId="4" xfId="8" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="9">
@@ -887,8 +887,11 @@
   </cellStyles>
   <dxfs count="31">
     <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
       <font>
-        <b/>
+        <b val="0"/>
         <i val="0"/>
         <strike val="0"/>
         <condense val="0"/>
@@ -897,28 +900,13 @@
         <shadow val="0"/>
         <u val="none"/>
         <vertAlign val="baseline"/>
-        <sz val="10"/>
+        <sz val="11"/>
         <color rgb="FF000000"/>
-        <name val="Helvetica Neue"/>
+        <name val="Calibri"/>
         <family val="2"/>
-        <scheme val="none"/>
+        <scheme val="minor"/>
       </font>
-      <numFmt numFmtId="1" formatCode="0"/>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top/>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <font>
@@ -931,386 +919,13 @@
         <shadow val="0"/>
         <u val="none"/>
         <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <name val="Helvetica Neue"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <numFmt numFmtId="1" formatCode="0"/>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <name val="Helvetica Neue"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <numFmt numFmtId="1" formatCode="0"/>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <name val="Helvetica Neue"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <numFmt numFmtId="1" formatCode="0"/>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="165" formatCode="_-&quot;$&quot;* #,##0.00_-;\-&quot;$&quot;* #,##0.00_-;_-&quot;$&quot;* &quot;-&quot;??_-;_-@_-"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <name val="Helvetica Neue"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <numFmt numFmtId="1" formatCode="0"/>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <name val="Helvetica Neue"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <numFmt numFmtId="1" formatCode="0"/>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <name val="Helvetica Neue"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <numFmt numFmtId="170" formatCode="_-&quot;$&quot;\ * #,##0.00_-;\-&quot;$&quot;\ * #,##0.00_-;_-&quot;$&quot;\ * &quot;-&quot;_-;_-@_-"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left/>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <name val="Helvetica Neue"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color theme="0"/>
+        <sz val="11"/>
+        <color theme="1"/>
         <name val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
       </font>
-      <numFmt numFmtId="1" formatCode="0"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="8"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top/>
-        <bottom/>
-      </border>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -1489,7 +1104,257 @@
       </border>
     </dxf>
     <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <name val="Helvetica Neue"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="1" formatCode="0"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top/>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <name val="Helvetica Neue"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="1" formatCode="0"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <name val="Helvetica Neue"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="1" formatCode="0"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <name val="Helvetica Neue"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="1" formatCode="0"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="165" formatCode="_-&quot;$&quot;* #,##0.00_-;\-&quot;$&quot;* #,##0.00_-;_-&quot;$&quot;* &quot;-&quot;??_-;_-@_-"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <name val="Helvetica Neue"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="1" formatCode="0"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <name val="Helvetica Neue"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="1" formatCode="0"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
     </dxf>
     <dxf>
       <font>
@@ -1502,13 +1367,112 @@
         <shadow val="0"/>
         <u val="none"/>
         <vertAlign val="baseline"/>
-        <sz val="11"/>
+        <sz val="10"/>
         <color rgb="FF000000"/>
-        <name val="Calibri"/>
+        <name val="Helvetica Neue"/>
         <family val="2"/>
-        <scheme val="minor"/>
+        <scheme val="none"/>
       </font>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <numFmt numFmtId="170" formatCode="_-&quot;$&quot;\ * #,##0.00_-;\-&quot;$&quot;\ * #,##0.00_-;_-&quot;$&quot;\ * &quot;-&quot;_-;_-@_-"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
     </dxf>
     <dxf>
       <font>
@@ -1521,13 +1485,49 @@
         <shadow val="0"/>
         <u val="none"/>
         <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <name val="Helvetica Neue"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="0"/>
         <name val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
       </font>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <numFmt numFmtId="1" formatCode="0"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="8"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top/>
+        <bottom/>
+      </border>
     </dxf>
   </dxfs>
   <tableStyles count="1" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16">
@@ -1740,60 +1740,60 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{8A94E3B6-9EAD-4329-8389-0ADCBCC848EA}" name="Tabla1" displayName="Tabla1" ref="A14:H42" totalsRowShown="0" headerRowDxfId="27" dataDxfId="25" headerRowBorderDxfId="26" tableBorderDxfId="24">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{8A94E3B6-9EAD-4329-8389-0ADCBCC848EA}" name="Tabla1" displayName="Tabla1" ref="A14:H42" totalsRowShown="0" headerRowDxfId="14" dataDxfId="12" headerRowBorderDxfId="13" tableBorderDxfId="11">
   <autoFilter ref="A14:H42" xr:uid="{8A94E3B6-9EAD-4329-8389-0ADCBCC848EA}"/>
   <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{520CA9FA-584B-4358-9B15-E654607E7AA3}" name="Código Interno" dataDxfId="23"/>
-    <tableColumn id="2" xr3:uid="{B5EE805F-D79D-4B18-9969-A438C10D73CB}" name="Código de Barra" dataDxfId="22">
+    <tableColumn id="1" xr3:uid="{520CA9FA-584B-4358-9B15-E654607E7AA3}" name="Código Interno" dataDxfId="10"/>
+    <tableColumn id="2" xr3:uid="{B5EE805F-D79D-4B18-9969-A438C10D73CB}" name="Código de Barra" dataDxfId="9">
       <calculatedColumnFormula>IFERROR(_xlfn.XLOOKUP(K15,Precios!K:K,Precios!I:I,0),"0")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{8E379099-A773-4C78-99DE-A30F428DCAA3}" name="Descripción del producto/servicio" dataDxfId="21"/>
-    <tableColumn id="5" xr3:uid="{3D35979A-292B-42DE-B9B7-4C01FAD4E4DB}" name="Cajas" dataDxfId="20"/>
-    <tableColumn id="6" xr3:uid="{1C8C5A17-73DF-4E24-BD8B-C3B44F70EC3B}" name="Piezas por Cj" dataDxfId="19"/>
-    <tableColumn id="7" xr3:uid="{4AC8BB4B-EFC3-40D6-BD2F-E267A391DA14}" name="Precio Unitario US$" dataDxfId="18"/>
-    <tableColumn id="8" xr3:uid="{8E18F1A5-A975-43AC-AC23-157590FF40C9}" name="Precio Caja US$" dataDxfId="17"/>
-    <tableColumn id="9" xr3:uid="{5EEA48C5-DAD6-467E-BE56-8D618AF7F476}" name="Precio Total" dataDxfId="16"/>
+    <tableColumn id="3" xr3:uid="{8E379099-A773-4C78-99DE-A30F428DCAA3}" name="Descripción del producto/servicio" dataDxfId="8"/>
+    <tableColumn id="5" xr3:uid="{3D35979A-292B-42DE-B9B7-4C01FAD4E4DB}" name="Cajas" dataDxfId="7"/>
+    <tableColumn id="6" xr3:uid="{1C8C5A17-73DF-4E24-BD8B-C3B44F70EC3B}" name="Piezas por Cj" dataDxfId="6"/>
+    <tableColumn id="7" xr3:uid="{4AC8BB4B-EFC3-40D6-BD2F-E267A391DA14}" name="Precio Unitario US$" dataDxfId="5"/>
+    <tableColumn id="8" xr3:uid="{8E18F1A5-A975-43AC-AC23-157590FF40C9}" name="Precio Caja US$" dataDxfId="4"/>
+    <tableColumn id="9" xr3:uid="{5EEA48C5-DAD6-467E-BE56-8D618AF7F476}" name="Precio Total" dataDxfId="3"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight16" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{8669CD56-B58B-4ACB-8B3C-F2934DCE7691}" name="Tabla2" displayName="Tabla2" ref="A1:F5" totalsRowShown="0" headerRowDxfId="30">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{8669CD56-B58B-4ACB-8B3C-F2934DCE7691}" name="Tabla2" displayName="Tabla2" ref="A1:F5" totalsRowShown="0" headerRowDxfId="2">
   <autoFilter ref="A1:F5" xr:uid="{8669CD56-B58B-4ACB-8B3C-F2934DCE7691}"/>
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{0D58B185-A9C1-48AD-B2F4-32DF9E217F13}" name="NIF:"/>
     <tableColumn id="2" xr3:uid="{33CBF84B-48C6-447A-BBF2-DD5AA8FCC61A}" name="Cliente"/>
     <tableColumn id="3" xr3:uid="{24888C6A-371D-47AF-9D61-4D5A564AB563}" name="DIRECCION"/>
-    <tableColumn id="4" xr3:uid="{54776D73-D261-4857-BA0D-C5404DB9B619}" name="Contacto:" dataDxfId="29"/>
+    <tableColumn id="4" xr3:uid="{54776D73-D261-4857-BA0D-C5404DB9B619}" name="Contacto:" dataDxfId="1"/>
     <tableColumn id="5" xr3:uid="{92F18AB8-E877-464C-B2B7-EB1E14CC628E}" name="NUMERO"/>
-    <tableColumn id="6" xr3:uid="{517F7E11-B7D8-4826-98B4-D4A8F078F50D}" name="LISTA_PRECIOS" dataDxfId="28"/>
+    <tableColumn id="6" xr3:uid="{517F7E11-B7D8-4826-98B4-D4A8F078F50D}" name="LISTA_PRECIOS" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{9A4FE505-CC4B-404E-AD0E-A96422E28D9D}" name="Tabla3" displayName="Tabla3" ref="A1:M11" totalsRowShown="0" headerRowDxfId="15" dataDxfId="14" tableBorderDxfId="13" dataCellStyle="Moneda [0]">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{9A4FE505-CC4B-404E-AD0E-A96422E28D9D}" name="Tabla3" displayName="Tabla3" ref="A1:M11" totalsRowShown="0" headerRowDxfId="30" dataDxfId="29" tableBorderDxfId="28" dataCellStyle="Moneda [0]">
   <autoFilter ref="A1:M11" xr:uid="{9A4FE505-CC4B-404E-AD0E-A96422E28D9D}"/>
   <tableColumns count="13">
-    <tableColumn id="1" xr3:uid="{DA0F2924-236B-47E9-A2A7-9191F873C793}" name="MARCA" dataDxfId="12"/>
-    <tableColumn id="2" xr3:uid="{D6ABD749-CE3A-429C-BE83-AC7C508C046F}" name="CODIGO" dataDxfId="11"/>
-    <tableColumn id="3" xr3:uid="{2839CEA5-BFD1-4AF4-9992-43115BB826C1}" name="Descripcion" dataDxfId="10"/>
-    <tableColumn id="4" xr3:uid="{66385BFB-7AC9-4F92-AEE8-3895D2EC51F5}" name="GRAMOS" dataDxfId="9"/>
-    <tableColumn id="5" xr3:uid="{791BE4D0-775A-4584-B7A9-A710D72CA463}" name="Precio CIF" dataDxfId="8" dataCellStyle="Moneda [0]"/>
-    <tableColumn id="6" xr3:uid="{7DC72C83-E4B3-4FA6-A4BB-7DFD7B7351DE}" name="Caja" dataDxfId="7" dataCellStyle="Moneda [0]"/>
-    <tableColumn id="7" xr3:uid="{E322D55A-4385-489C-B408-E5F854A495AF}" name="Pallet" dataDxfId="6" dataCellStyle="Moneda [0]"/>
-    <tableColumn id="11" xr3:uid="{B97156C5-49D3-4846-A5C8-ABD0A02AAA8D}" name="Precio CJ" dataDxfId="5">
+    <tableColumn id="1" xr3:uid="{DA0F2924-236B-47E9-A2A7-9191F873C793}" name="MARCA" dataDxfId="27"/>
+    <tableColumn id="2" xr3:uid="{D6ABD749-CE3A-429C-BE83-AC7C508C046F}" name="CODIGO" dataDxfId="26"/>
+    <tableColumn id="3" xr3:uid="{2839CEA5-BFD1-4AF4-9992-43115BB826C1}" name="Descripcion" dataDxfId="25"/>
+    <tableColumn id="4" xr3:uid="{66385BFB-7AC9-4F92-AEE8-3895D2EC51F5}" name="GRAMOS" dataDxfId="24"/>
+    <tableColumn id="5" xr3:uid="{791BE4D0-775A-4584-B7A9-A710D72CA463}" name="Precio CIF" dataDxfId="23" dataCellStyle="Moneda [0]"/>
+    <tableColumn id="6" xr3:uid="{7DC72C83-E4B3-4FA6-A4BB-7DFD7B7351DE}" name="Caja" dataDxfId="22" dataCellStyle="Moneda [0]"/>
+    <tableColumn id="7" xr3:uid="{E322D55A-4385-489C-B408-E5F854A495AF}" name="Pallet" dataDxfId="21" dataCellStyle="Moneda [0]"/>
+    <tableColumn id="11" xr3:uid="{B97156C5-49D3-4846-A5C8-ABD0A02AAA8D}" name="Precio CJ" dataDxfId="20">
       <calculatedColumnFormula>E2*F2</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="12" xr3:uid="{2C02D87E-8CB1-49F8-A5BE-03855A6C1E9B}" name="COD BARRAS" dataDxfId="4"/>
-    <tableColumn id="13" xr3:uid="{E5AD99A8-D6B8-4E4D-B228-7FB94061B422}" name="LISTA_PRECIOS" dataDxfId="3" dataCellStyle="Moneda [0]"/>
-    <tableColumn id="14" xr3:uid="{51631B47-0651-4FAD-9063-AA561FBD4C48}" name="Clave" dataDxfId="2" dataCellStyle="Moneda [0]">
+    <tableColumn id="12" xr3:uid="{2C02D87E-8CB1-49F8-A5BE-03855A6C1E9B}" name="COD BARRAS" dataDxfId="19"/>
+    <tableColumn id="13" xr3:uid="{E5AD99A8-D6B8-4E4D-B228-7FB94061B422}" name="LISTA_PRECIOS" dataDxfId="18" dataCellStyle="Moneda [0]"/>
+    <tableColumn id="14" xr3:uid="{51631B47-0651-4FAD-9063-AA561FBD4C48}" name="Clave" dataDxfId="17" dataCellStyle="Moneda [0]">
       <calculatedColumnFormula>_xlfn.CONCAT(Tabla3[[#This Row],[CODIGO]],Tabla3[[#This Row],[LISTA_PRECIOS]])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="16" xr3:uid="{AC660C86-F1B8-4D6F-B5EA-B71D403A6C74}" name="Columna1" dataDxfId="1" dataCellStyle="Moneda [0]"/>
-    <tableColumn id="8" xr3:uid="{AC200EC2-556C-E346-8A2C-D4CB607D1887}" name="ORIGEN" dataDxfId="0" dataCellStyle="Moneda [0]"/>
+    <tableColumn id="16" xr3:uid="{AC660C86-F1B8-4D6F-B5EA-B71D403A6C74}" name="Columna1" dataDxfId="16" dataCellStyle="Moneda [0]"/>
+    <tableColumn id="8" xr3:uid="{AC200EC2-556C-E346-8A2C-D4CB607D1887}" name="ORIGEN" dataDxfId="15" dataCellStyle="Moneda [0]"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2109,9 +2109,9 @@
       <c r="F2" s="40"/>
       <c r="G2" s="40"/>
       <c r="H2" s="40"/>
-      <c r="I2" s="82"/>
-      <c r="K2" s="78"/>
-      <c r="L2" s="78"/>
+      <c r="I2" s="83"/>
+      <c r="K2" s="79"/>
+      <c r="L2" s="79"/>
       <c r="M2" s="33"/>
     </row>
     <row r="3" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -2123,7 +2123,7 @@
       <c r="F3" s="41"/>
       <c r="G3" s="41"/>
       <c r="H3" s="41"/>
-      <c r="I3" s="82"/>
+      <c r="I3" s="83"/>
     </row>
     <row r="4" spans="1:13" ht="16" x14ac:dyDescent="0.2">
       <c r="A4" s="42" t="s">
@@ -2140,7 +2140,7 @@
         <v>6</v>
       </c>
       <c r="H4" s="46"/>
-      <c r="I4" s="82"/>
+      <c r="I4" s="83"/>
     </row>
     <row r="5" spans="1:13" ht="16" x14ac:dyDescent="0.2">
       <c r="A5" s="42" t="s">
@@ -2160,22 +2160,22 @@
         <v>18</v>
       </c>
       <c r="H5" s="36"/>
-      <c r="I5" s="82"/>
+      <c r="I5" s="83"/>
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A6" s="42" t="s">
         <v>1</v>
       </c>
-      <c r="B6" s="83" t="s">
+      <c r="B6" s="84" t="s">
         <v>2</v>
       </c>
-      <c r="C6" s="83"/>
+      <c r="C6" s="84"/>
       <c r="D6" s="41"/>
       <c r="E6" s="41"/>
       <c r="F6" s="42"/>
       <c r="G6" s="48"/>
       <c r="H6" s="41"/>
-      <c r="I6" s="82"/>
+      <c r="I6" s="83"/>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A7" s="42" t="s">
@@ -2190,7 +2190,7 @@
       <c r="F7" s="50"/>
       <c r="G7" s="36"/>
       <c r="H7" s="36"/>
-      <c r="I7" s="82"/>
+      <c r="I7" s="83"/>
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A8" s="42"/>
@@ -2203,7 +2203,7 @@
       <c r="F8" s="51"/>
       <c r="G8" s="43"/>
       <c r="H8" s="48"/>
-      <c r="I8" s="82"/>
+      <c r="I8" s="83"/>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A9" s="41"/>
@@ -2214,17 +2214,17 @@
       <c r="F9" s="41"/>
       <c r="G9" s="41"/>
       <c r="H9" s="41"/>
-      <c r="I9" s="82"/>
+      <c r="I9" s="83"/>
     </row>
     <row r="10" spans="1:13" ht="19" x14ac:dyDescent="0.2">
       <c r="A10" s="52" t="s">
         <v>7</v>
       </c>
-      <c r="B10" s="80" t="str">
+      <c r="B10" s="81" t="str">
         <f>_xlfn.XLOOKUP(B13,Clientes!A:A,Clientes!B:B,0)</f>
         <v>Bravo</v>
       </c>
-      <c r="C10" s="80"/>
+      <c r="C10" s="81"/>
       <c r="D10" s="53"/>
       <c r="E10" s="53"/>
       <c r="F10" s="52" t="s">
@@ -2232,18 +2232,18 @@
       </c>
       <c r="G10" s="54"/>
       <c r="H10" s="53"/>
-      <c r="I10" s="82"/>
+      <c r="I10" s="83"/>
     </row>
     <row r="11" spans="1:13" ht="16" x14ac:dyDescent="0.2">
       <c r="A11" s="52" t="s">
         <v>4</v>
       </c>
-      <c r="B11" s="79" t="str">
+      <c r="B11" s="80" t="str">
         <f>_xlfn.XLOOKUP(B13,Clientes!A:A,Clientes!C:C,0)</f>
         <v>Calle Central, Zona Industrial de Herrera, Santo Domingo</v>
       </c>
-      <c r="C11" s="79"/>
-      <c r="D11" s="79"/>
+      <c r="C11" s="80"/>
+      <c r="D11" s="80"/>
       <c r="E11" s="55"/>
       <c r="F11" s="52" t="s">
         <v>17</v>
@@ -2253,7 +2253,7 @@
         <v>809-227-2605</v>
       </c>
       <c r="H11" s="56"/>
-      <c r="I11" s="82"/>
+      <c r="I11" s="83"/>
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A12" s="52" t="s">
@@ -2271,7 +2271,7 @@
         <v>AUBRAVO</v>
       </c>
       <c r="H12" s="61"/>
-      <c r="I12" s="82"/>
+      <c r="I12" s="83"/>
     </row>
     <row r="13" spans="1:13" ht="28.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="52" t="s">
@@ -2280,13 +2280,13 @@
       <c r="B13" s="59">
         <v>125020</v>
       </c>
-      <c r="C13" s="81"/>
-      <c r="D13" s="81"/>
+      <c r="C13" s="82"/>
+      <c r="D13" s="82"/>
       <c r="E13" s="59"/>
       <c r="F13" s="59"/>
       <c r="G13" s="57"/>
       <c r="H13" s="62"/>
-      <c r="I13" s="82"/>
+      <c r="I13" s="83"/>
     </row>
     <row r="14" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A14" s="63" t="s">
@@ -2313,7 +2313,7 @@
       <c r="H14" s="63" t="s">
         <v>11</v>
       </c>
-      <c r="I14" s="82"/>
+      <c r="I14" s="83"/>
       <c r="K14" s="34" t="s">
         <v>68</v>
       </c>
@@ -2349,7 +2349,7 @@
         <f>G15*D15</f>
         <v>15774.8</v>
       </c>
-      <c r="I15" s="82"/>
+      <c r="I15" s="83"/>
       <c r="K15" s="2" t="str">
         <f>_xlfn.CONCAT(Tabla1[[#This Row],[Código Interno]],$G$12)</f>
         <v>504757AUBRAVO</v>
@@ -2386,7 +2386,7 @@
         <f>G16*D16</f>
         <v>1427.9999999999998</v>
       </c>
-      <c r="I16" s="82"/>
+      <c r="I16" s="83"/>
       <c r="K16" s="2" t="str">
         <f>_xlfn.CONCAT(Tabla1[[#This Row],[Código Interno]],$G$12)</f>
         <v>24184AUBRAVO</v>
@@ -2423,7 +2423,7 @@
         <f>G17*D17</f>
         <v>2855.9999999999995</v>
       </c>
-      <c r="I17" s="82"/>
+      <c r="I17" s="83"/>
       <c r="K17" s="2" t="str">
         <f>_xlfn.CONCAT(Tabla1[[#This Row],[Código Interno]],$G$12)</f>
         <v>1233AUBRAVO</v>
@@ -2460,7 +2460,7 @@
         <f>G18*D18</f>
         <v>2855.9999999999995</v>
       </c>
-      <c r="I18" s="82"/>
+      <c r="I18" s="83"/>
       <c r="K18" s="2" t="str">
         <f>_xlfn.CONCAT(Tabla1[[#This Row],[Código Interno]],$G$12)</f>
         <v>505252AUBRAVO</v>
@@ -2475,7 +2475,7 @@
       <c r="F19" s="35"/>
       <c r="G19" s="69"/>
       <c r="H19" s="70"/>
-      <c r="I19" s="82"/>
+      <c r="I19" s="83"/>
       <c r="K19" s="2" t="str">
         <f>_xlfn.CONCAT(Tabla1[[#This Row],[Código Interno]],$G$12)</f>
         <v>AUBRAVO</v>
@@ -2490,7 +2490,7 @@
       <c r="F20" s="35"/>
       <c r="G20" s="69"/>
       <c r="H20" s="70"/>
-      <c r="I20" s="82"/>
+      <c r="I20" s="83"/>
       <c r="K20" s="2" t="str">
         <f>_xlfn.CONCAT(Tabla1[[#This Row],[Código Interno]],$G$12)</f>
         <v>AUBRAVO</v>
@@ -2505,7 +2505,7 @@
       <c r="F21" s="35"/>
       <c r="G21" s="69"/>
       <c r="H21" s="70"/>
-      <c r="I21" s="82"/>
+      <c r="I21" s="83"/>
       <c r="K21" s="2" t="str">
         <f>_xlfn.CONCAT(Tabla1[[#This Row],[Código Interno]],$G$12)</f>
         <v>AUBRAVO</v>
@@ -2520,7 +2520,7 @@
       <c r="F22" s="35"/>
       <c r="G22" s="69"/>
       <c r="H22" s="70"/>
-      <c r="I22" s="82"/>
+      <c r="I22" s="83"/>
       <c r="K22" s="2" t="str">
         <f>_xlfn.CONCAT(Tabla1[[#This Row],[Código Interno]],$G$12)</f>
         <v>AUBRAVO</v>
@@ -2535,7 +2535,7 @@
       <c r="F23" s="35"/>
       <c r="G23" s="69"/>
       <c r="H23" s="70"/>
-      <c r="I23" s="82"/>
+      <c r="I23" s="83"/>
       <c r="K23" s="2" t="str">
         <f>_xlfn.CONCAT(Tabla1[[#This Row],[Código Interno]],$G$12)</f>
         <v>AUBRAVO</v>
@@ -2550,7 +2550,7 @@
       <c r="F24" s="35"/>
       <c r="G24" s="69"/>
       <c r="H24" s="70"/>
-      <c r="I24" s="82"/>
+      <c r="I24" s="83"/>
       <c r="K24" s="2" t="str">
         <f>_xlfn.CONCAT(Tabla1[[#This Row],[Código Interno]],$G$12)</f>
         <v>AUBRAVO</v>
@@ -2565,7 +2565,7 @@
       <c r="F25" s="35"/>
       <c r="G25" s="69"/>
       <c r="H25" s="70"/>
-      <c r="I25" s="82"/>
+      <c r="I25" s="83"/>
       <c r="K25" s="2" t="str">
         <f>_xlfn.CONCAT(Tabla1[[#This Row],[Código Interno]],$G$12)</f>
         <v>AUBRAVO</v>
@@ -2580,7 +2580,7 @@
       <c r="F26" s="35"/>
       <c r="G26" s="69"/>
       <c r="H26" s="70"/>
-      <c r="I26" s="82"/>
+      <c r="I26" s="83"/>
       <c r="K26" s="2" t="str">
         <f>_xlfn.CONCAT(Tabla1[[#This Row],[Código Interno]],$G$12)</f>
         <v>AUBRAVO</v>
@@ -2595,7 +2595,7 @@
       <c r="F27" s="35"/>
       <c r="G27" s="69"/>
       <c r="H27" s="70"/>
-      <c r="I27" s="82"/>
+      <c r="I27" s="83"/>
       <c r="K27" s="2" t="str">
         <f>_xlfn.CONCAT(Tabla1[[#This Row],[Código Interno]],$G$12)</f>
         <v>AUBRAVO</v>
@@ -2610,7 +2610,7 @@
       <c r="F28" s="35"/>
       <c r="G28" s="69"/>
       <c r="H28" s="70"/>
-      <c r="I28" s="82"/>
+      <c r="I28" s="83"/>
       <c r="K28" s="2" t="str">
         <f>_xlfn.CONCAT(Tabla1[[#This Row],[Código Interno]],$G$12)</f>
         <v>AUBRAVO</v>
@@ -2625,7 +2625,7 @@
       <c r="F29" s="35"/>
       <c r="G29" s="69"/>
       <c r="H29" s="70"/>
-      <c r="I29" s="82"/>
+      <c r="I29" s="83"/>
       <c r="K29" s="2" t="str">
         <f>_xlfn.CONCAT(Tabla1[[#This Row],[Código Interno]],$G$12)</f>
         <v>AUBRAVO</v>
@@ -2640,7 +2640,7 @@
       <c r="F30" s="35"/>
       <c r="G30" s="69"/>
       <c r="H30" s="70"/>
-      <c r="I30" s="82"/>
+      <c r="I30" s="83"/>
       <c r="K30" s="2" t="str">
         <f>_xlfn.CONCAT(Tabla1[[#This Row],[Código Interno]],$G$12)</f>
         <v>AUBRAVO</v>
@@ -2655,7 +2655,7 @@
       <c r="F31" s="35"/>
       <c r="G31" s="69"/>
       <c r="H31" s="70"/>
-      <c r="I31" s="82"/>
+      <c r="I31" s="83"/>
       <c r="K31" s="2" t="str">
         <f>_xlfn.CONCAT(Tabla1[[#This Row],[Código Interno]],$G$12)</f>
         <v>AUBRAVO</v>
@@ -2670,7 +2670,7 @@
       <c r="F32" s="35"/>
       <c r="G32" s="69"/>
       <c r="H32" s="70"/>
-      <c r="I32" s="82"/>
+      <c r="I32" s="83"/>
       <c r="K32" s="2" t="str">
         <f>_xlfn.CONCAT(Tabla1[[#This Row],[Código Interno]],$G$12)</f>
         <v>AUBRAVO</v>
@@ -2685,7 +2685,7 @@
       <c r="F33" s="35"/>
       <c r="G33" s="69"/>
       <c r="H33" s="70"/>
-      <c r="I33" s="82"/>
+      <c r="I33" s="83"/>
       <c r="K33" s="2" t="str">
         <f>_xlfn.CONCAT(Tabla1[[#This Row],[Código Interno]],$G$12)</f>
         <v>AUBRAVO</v>
@@ -2700,7 +2700,7 @@
       <c r="F34" s="35"/>
       <c r="G34" s="69"/>
       <c r="H34" s="70"/>
-      <c r="I34" s="82"/>
+      <c r="I34" s="83"/>
       <c r="K34" s="2" t="str">
         <f>_xlfn.CONCAT(Tabla1[[#This Row],[Código Interno]],$G$12)</f>
         <v>AUBRAVO</v>
@@ -2715,7 +2715,7 @@
       <c r="F35" s="35"/>
       <c r="G35" s="69"/>
       <c r="H35" s="70"/>
-      <c r="I35" s="82"/>
+      <c r="I35" s="83"/>
       <c r="K35" s="2" t="str">
         <f>_xlfn.CONCAT(Tabla1[[#This Row],[Código Interno]],$G$12)</f>
         <v>AUBRAVO</v>
@@ -2730,7 +2730,7 @@
       <c r="F36" s="35"/>
       <c r="G36" s="69"/>
       <c r="H36" s="70"/>
-      <c r="I36" s="82"/>
+      <c r="I36" s="83"/>
       <c r="K36" s="2" t="str">
         <f>_xlfn.CONCAT(Tabla1[[#This Row],[Código Interno]],$G$12)</f>
         <v>AUBRAVO</v>
@@ -2745,7 +2745,7 @@
       <c r="F37" s="35"/>
       <c r="G37" s="69"/>
       <c r="H37" s="70"/>
-      <c r="I37" s="82"/>
+      <c r="I37" s="83"/>
       <c r="K37" s="2" t="str">
         <f>_xlfn.CONCAT(Tabla1[[#This Row],[Código Interno]],$G$12)</f>
         <v>AUBRAVO</v>
@@ -2760,7 +2760,7 @@
       <c r="F38" s="35"/>
       <c r="G38" s="69"/>
       <c r="H38" s="70"/>
-      <c r="I38" s="82"/>
+      <c r="I38" s="83"/>
       <c r="K38" s="2" t="str">
         <f>_xlfn.CONCAT(Tabla1[[#This Row],[Código Interno]],$G$12)</f>
         <v>AUBRAVO</v>
@@ -2775,7 +2775,7 @@
       <c r="F39" s="35"/>
       <c r="G39" s="69"/>
       <c r="H39" s="67"/>
-      <c r="I39" s="82"/>
+      <c r="I39" s="83"/>
       <c r="K39" s="2" t="str">
         <f>_xlfn.CONCAT(Tabla1[[#This Row],[Código Interno]],$G$12)</f>
         <v>AUBRAVO</v>
@@ -2790,7 +2790,7 @@
       <c r="F40" s="35"/>
       <c r="G40" s="69"/>
       <c r="H40" s="67"/>
-      <c r="I40" s="82"/>
+      <c r="I40" s="83"/>
       <c r="K40" s="2" t="str">
         <f>_xlfn.CONCAT(Tabla1[[#This Row],[Código Interno]],$G$12)</f>
         <v>AUBRAVO</v>
@@ -2805,7 +2805,7 @@
       <c r="F41" s="35"/>
       <c r="G41" s="69"/>
       <c r="H41" s="67"/>
-      <c r="I41" s="82"/>
+      <c r="I41" s="83"/>
       <c r="K41" s="2" t="str">
         <f>_xlfn.CONCAT(Tabla1[[#This Row],[Código Interno]],$G$12)</f>
         <v>AUBRAVO</v>
@@ -2820,7 +2820,7 @@
       <c r="F42" s="35"/>
       <c r="G42" s="69"/>
       <c r="H42" s="67"/>
-      <c r="I42" s="82"/>
+      <c r="I42" s="83"/>
       <c r="K42" s="2" t="str">
         <f>_xlfn.CONCAT(Tabla1[[#This Row],[Código Interno]],$G$12)</f>
         <v>AUBRAVO</v>
@@ -2831,7 +2831,7 @@
       <c r="C43" s="71"/>
       <c r="E43" s="52"/>
       <c r="F43" s="52"/>
-      <c r="I43" s="82"/>
+      <c r="I43" s="83"/>
     </row>
     <row r="44" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A44" s="41"/>
@@ -2843,7 +2843,7 @@
         <v>13</v>
       </c>
       <c r="H44" s="74"/>
-      <c r="I44" s="82"/>
+      <c r="I44" s="83"/>
     </row>
     <row r="45" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A45" s="75" t="s">
@@ -2860,7 +2860,7 @@
         <f>SUM(H15:H42)</f>
         <v>22914.799999999999</v>
       </c>
-      <c r="I45" s="82"/>
+      <c r="I45" s="83"/>
     </row>
     <row r="46" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A46" s="76" t="s">
@@ -2876,7 +2876,7 @@
       <c r="H46" s="31" t="s">
         <v>16</v>
       </c>
-      <c r="I46" s="82"/>
+      <c r="I46" s="83"/>
     </row>
     <row r="47" spans="1:11" ht="17" x14ac:dyDescent="0.2">
       <c r="A47" s="77"/>
@@ -2891,7 +2891,7 @@
       <c r="H47" s="31" t="s">
         <v>42</v>
       </c>
-      <c r="I47" s="82"/>
+      <c r="I47" s="83"/>
     </row>
     <row r="48" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
       <c r="A48" s="16"/>
@@ -2902,7 +2902,7 @@
       <c r="F48" s="14"/>
       <c r="G48" s="14"/>
       <c r="H48" s="14"/>
-      <c r="I48" s="82"/>
+      <c r="I48" s="83"/>
     </row>
     <row r="51" spans="3:3" hidden="1" x14ac:dyDescent="0.2">
       <c r="C51" s="1"/>
@@ -3131,7 +3131,7 @@
       <c r="L2" s="29" t="s">
         <v>60</v>
       </c>
-      <c r="M2" s="84" t="s">
+      <c r="M2" s="78" t="s">
         <v>73</v>
       </c>
     </row>
@@ -3174,7 +3174,7 @@
       <c r="L3" s="29" t="s">
         <v>60</v>
       </c>
-      <c r="M3" s="84" t="s">
+      <c r="M3" s="78" t="s">
         <v>73</v>
       </c>
     </row>
@@ -3217,7 +3217,7 @@
       <c r="L4" s="29" t="s">
         <v>60</v>
       </c>
-      <c r="M4" s="84" t="s">
+      <c r="M4" s="78" t="s">
         <v>73</v>
       </c>
     </row>
@@ -3260,7 +3260,7 @@
       <c r="L5" s="29" t="s">
         <v>60</v>
       </c>
-      <c r="M5" s="84" t="s">
+      <c r="M5" s="78" t="s">
         <v>73</v>
       </c>
     </row>
@@ -3303,7 +3303,7 @@
       <c r="L6" s="29" t="s">
         <v>60</v>
       </c>
-      <c r="M6" s="84" t="s">
+      <c r="M6" s="78" t="s">
         <v>73</v>
       </c>
     </row>
@@ -3346,7 +3346,7 @@
       <c r="L7" s="10" t="s">
         <v>53</v>
       </c>
-      <c r="M7" s="84" t="s">
+      <c r="M7" s="78" t="s">
         <v>73</v>
       </c>
     </row>
@@ -3389,7 +3389,7 @@
       <c r="L8" s="10" t="s">
         <v>53</v>
       </c>
-      <c r="M8" s="84" t="s">
+      <c r="M8" s="78" t="s">
         <v>73</v>
       </c>
     </row>
@@ -3432,7 +3432,7 @@
       <c r="L9" s="10" t="s">
         <v>53</v>
       </c>
-      <c r="M9" s="84" t="s">
+      <c r="M9" s="78" t="s">
         <v>73</v>
       </c>
     </row>
@@ -3475,7 +3475,7 @@
       <c r="L10" s="10" t="s">
         <v>53</v>
       </c>
-      <c r="M10" s="84" t="s">
+      <c r="M10" s="78" t="s">
         <v>73</v>
       </c>
     </row>
@@ -3518,7 +3518,7 @@
       <c r="L11" s="10" t="s">
         <v>53</v>
       </c>
-      <c r="M11" s="84" t="s">
+      <c r="M11" s="78" t="s">
         <v>73</v>
       </c>
     </row>

</xml_diff>